<commit_message>
feat: add regional chili dataset files and update preprocessing and deployment configurations
</commit_message>
<xml_diff>
--- a/clean_data/Aceh_Cabai Merah Besar.xlsx
+++ b/clean_data/Aceh_Cabai Merah Besar.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1707"/>
+  <dimension ref="A1:B1708"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14065,7 +14065,7 @@
         <v>46209</v>
       </c>
       <c r="B1704" t="n">
-        <v>40300</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="1705">
@@ -14073,7 +14073,7 @@
         <v>46210</v>
       </c>
       <c r="B1705" t="n">
-        <v>40300</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="1706">
@@ -14081,7 +14081,7 @@
         <v>46211</v>
       </c>
       <c r="B1706" t="n">
-        <v>40500</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="1707">
@@ -14089,7 +14089,15 @@
         <v>46212</v>
       </c>
       <c r="B1707" t="n">
-        <v>40300</v>
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B1708" t="n">
+        <v>35700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>